<commit_message>
Update the entropy logic
</commit_message>
<xml_diff>
--- a/tabular/refseq-core/ifnl-refseq-side-data.xlsx
+++ b/tabular/refseq-core/ifnl-refseq-side-data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10311"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10308"/>
   <workbookPr date1904="1" showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/robertgifford/Projects/host/IFNL-Evolution/tabular/refseq-core/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rob/Projects/host/IFNL-Evolution/tabular/refseq-core/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B940E404-2EA1-6D47-AF65-0E429FD8F09E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DF303C9-C5A9-3642-90B9-F7C11DD277B5}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17680" yWindow="5960" windowWidth="28060" windowHeight="17540" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="940" yWindow="500" windowWidth="27860" windowHeight="17500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="A+B" sheetId="2" r:id="rId1"/>

</xml_diff>